<commit_message>
feat(gms-subseq): keep sub-sequence running on cancel and restore on password cancel
- 서브시퀀스 진행 중 [취소] 클릭 시 즉시 강제 종료하지 않고 백그라운드 진행 유지
- 비밀번호 화면에서 [취소] 시 원래 서브시퀀스 진행 화면 및 패널 100% 안전 복원
- 비밀번호 확인 통과 시에만 window.stopAllSubSequences()로 완전 종료 및 복귀 처리
- 배관도 밸브(30종) 및 아날로그 센서(13종) 데이터 전 장비 동기화 및 4단계 fallback 복구
- pc-app과 mobile-app www 리소스 최신 상태 양방향 동기화
</commit_message>
<xml_diff>
--- a/projects/plc-monitoring-v1/GMS_전체_자동진행_시퀀스_알람_검증_체크시트.xlsx
+++ b/projects/plc-monitoring-v1/GMS_전체_자동진행_시퀀스_알람_검증_체크시트.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19종_시퀀스_알람_총괄요약" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="전체_알람_전수검증_체크시트" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시뮬레이션_통합검증_체크시트" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'전체_알람_전수검증_체크시트'!$A$3:$N$177</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'시뮬레이션_통합검증_체크시트'!$A$3:$J$29</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,8 +74,24 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -116,6 +134,12 @@
         <bgColor rgb="000284C7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -143,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -177,6 +201,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -545,7 +584,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -1321,7 +1360,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N177"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -13253,4 +13292,1393 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  🎯 GMS 실감형 운전자 조작 &amp; 전구간 시나리오 통합 검증 체크시트 (Driver Simulation Check Sheet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>대분류 (그룹)</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>검증 시험 항목</t>
+        </is>
+      </c>
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>운전자 조작 행위 (Action)</t>
+        </is>
+      </c>
+      <c r="E3" s="16" t="inlineStr">
+        <is>
+          <t>옵션 및 시스템 조건</t>
+        </is>
+      </c>
+      <c r="F3" s="16" t="inlineStr">
+        <is>
+          <t>정상 판정 기준 (Expected Result)</t>
+        </is>
+      </c>
+      <c r="G3" s="16" t="inlineStr">
+        <is>
+          <t>EMNG SHUT-DOWN / 취소 연동</t>
+        </is>
+      </c>
+      <c r="H3" s="16" t="inlineStr">
+        <is>
+          <t>배속 지원</t>
+        </is>
+      </c>
+      <c r="I3" s="16" t="inlineStr">
+        <is>
+          <t>시뮬레이션 검증</t>
+        </is>
+      </c>
+      <c r="J3" s="16" t="inlineStr">
+        <is>
+          <t>최종 판정</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>화면전환/보안</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>유지보수 화면 전환 및 [취소] 키 복귀</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>유지보수 버튼 클릭 ➔ 비밀번호 입력창 진입 ➔ [취소] 클릭</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>유지보수 진입 비밀번호 옵션 적용</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>비밀번호 창 닫히고 이전 메인 관제 화면으로 100% 정상 복귀</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>취소 키 원복 안전 검증</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J4" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>화면전환/보안</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>조작자 비밀번호 정상 인증 승인</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>비밀번호 창 재진입 ➔ 가상 키패드 4-3-2-1 타이핑 ➔ [확인] 클릭</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="inlineStr">
+        <is>
+          <t>마스터 계정 인증 (MASTER/4321)</t>
+        </is>
+      </c>
+      <c r="F5" s="18" t="inlineStr">
+        <is>
+          <t>비밀번호 인증 통과 후 [A] 유지보수 조작 패널 정상 진입</t>
+        </is>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>인증 통과 후 조작 활성화</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J5" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>화면전환/보안</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>비밀번호 옵션 미적용 시 직행 검증</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>비밀번호 옵션 [미적용] 변경 ➔ 메뉴 클릭</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>비밀번호 적용 옵션: 미적용(OFF)</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>비밀번호 입력 팝업 없이 해당 화면으로 즉시 직행 진입</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>게이트 우회 동작 검증</t>
+        </is>
+      </c>
+      <c r="H6" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J6" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>안전인터락</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>시퀀스 가동 중 [취소] 안전 복귀</t>
+        </is>
+      </c>
+      <c r="D7" s="18" t="inlineStr">
+        <is>
+          <t>1P 시퀀스 가동(VN1/PNV 밸브 Open) 중 ➔ [취소] 클릭</t>
+        </is>
+      </c>
+      <c r="E7" s="18" t="inlineStr">
+        <is>
+          <t>1P 자동진행 중</t>
+        </is>
+      </c>
+      <c r="F7" s="18" t="inlineStr">
+        <is>
+          <t>시퀀스 즉시 중단 ➔ 가동 중 밸브 안전 CLOSE ➔ 대기 복귀</t>
+        </is>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>필수 취소 안전 복귀</t>
+        </is>
+      </c>
+      <c r="H7" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>안전인터락</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>비상 [EMNG SHUT-DOWN] 인터락</t>
+        </is>
+      </c>
+      <c r="D8" s="18" t="inlineStr">
+        <is>
+          <t>공정 진행 또는 화면 전환 후 ➔ [SHUT-DOWN] 클릭</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>SHUT-DOWN 비상 운전 모드</t>
+        </is>
+      </c>
+      <c r="F8" s="18" t="inlineStr">
+        <is>
+          <t>경보 발생 ➔ 전 밸브(19종) 즉시 강제 CLOSE ➔ Cylinder Status IDLE 리셋</t>
+        </is>
+      </c>
+      <c r="G8" s="18" t="inlineStr">
+        <is>
+          <t>필수 비상 SHUT-DOWN TEST</t>
+        </is>
+      </c>
+      <c r="H8" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J8" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>안전인터락</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>수동조작 상태유지 옵션 연동</t>
+        </is>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>수동밸브 조작 중 취소 시 열림 상태 유지 여부 판정</t>
+        </is>
+      </c>
+      <c r="E9" s="18" t="inlineStr">
+        <is>
+          <t>수동조작 상태 유지: 적용 vs 미적용</t>
+        </is>
+      </c>
+      <c r="F9" s="18" t="inlineStr">
+        <is>
+          <t>적용 시 밸브 유지 퇴장 / 미적용 시 강제 차단 확인 팝업 호출</t>
+        </is>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>상태 유지 옵션 연동</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J9" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>시퀀스편집</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>시퀀스 순서 재배치 및 삭제 편집</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>Main 시퀀스 편집기 호출 ➔ -VT 삭제 및 3P 위치 변경 ➔ 저장</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>Main 시퀀스 에디터 모달</t>
+        </is>
+      </c>
+      <c r="F10" s="18" t="inlineStr">
+        <is>
+          <t>새 순서에 맞춰 상단 스텝 배지 재배열 및 변경된 순서대로 진행</t>
+        </is>
+      </c>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>순서 동적 편집 검증</t>
+        </is>
+      </c>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J10" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>시퀀스편집</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>시퀀스 순서 기본값 안전 리셋</t>
+        </is>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>편집기 내 [초기화] 클릭 ➔ 17단계 표준 순서 복원</t>
+        </is>
+      </c>
+      <c r="E11" s="18" t="inlineStr">
+        <is>
+          <t>표준 순서: IDLE➔Puls➔1P➔-L...➔Service</t>
+        </is>
+      </c>
+      <c r="F11" s="18" t="inlineStr">
+        <is>
+          <t>표준 시퀀스 순서로 100% 원복 및 배지 동기화</t>
+        </is>
+      </c>
+      <c r="G11" s="18" t="inlineStr">
+        <is>
+          <t>편집 복구 안전 검증</t>
+        </is>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J11" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>옵션테이블</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>VT 사용 옵션 분기 검증</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>-L 감압시험 완료 후 다음 공정 분기 판정</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>VT 사용 옵션: 적용(ON) vs 미적용(OFF)</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>적용 시 -VT 고진공 시험 진행 / 미적용 시 2P 배관청소 직행</t>
+        </is>
+      </c>
+      <c r="G12" s="18" t="inlineStr">
+        <is>
+          <t>동적 분기 검증</t>
+        </is>
+      </c>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J12" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>옵션테이블</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>Bypass 사용 옵션 분기 검증</t>
+        </is>
+      </c>
+      <c r="D13" s="18" t="inlineStr">
+        <is>
+          <t>용기교체(CC) 완료 후 Bypass 진행 여부 판정</t>
+        </is>
+      </c>
+      <c r="E13" s="18" t="inlineStr">
+        <is>
+          <t>Bypass 사용 옵션: 적용 vs 미적용</t>
+        </is>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>적용 시 Bypass 시퀀스 가동 / 미적용 시 3P로 즉시 스킵</t>
+        </is>
+      </c>
+      <c r="G13" s="18" t="inlineStr">
+        <is>
+          <t>동적 분기 검증</t>
+        </is>
+      </c>
+      <c r="H13" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J13" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>옵션테이블</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>1P 4종 서브시퀀스 개별 사용 여부</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>1P(Vent/2차Purge/Pumping/1차Purge) 개별 On/Off</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>1P 서브시퀀스 개별 토글</t>
+        </is>
+      </c>
+      <c r="F14" s="18" t="inlineStr">
+        <is>
+          <t>적용된 서브시퀀스만 정해진 순서대로 체인 실행, 미적용은 건너뜀</t>
+        </is>
+      </c>
+      <c r="G14" s="18" t="inlineStr">
+        <is>
+          <t>1P 체인 동적 연동</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J14" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>옵션테이블</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>가압시험 완료 후 Puls Vent 옵션</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>+L 가압시험 완료 후 Puls 2 진행 여부 판정</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Puls Vent 옵션: 적용 vs 미적용</t>
+        </is>
+      </c>
+      <c r="F15" s="18" t="inlineStr">
+        <is>
+          <t>적용 시 Puls 2 실행 후 4P / 미적용 시 즉시 4P 진입</t>
+        </is>
+      </c>
+      <c r="G15" s="18" t="inlineStr">
+        <is>
+          <t>후속 펄스 옵션 검증</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I15" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J15" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>옵션테이블</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>GC Type (2B1P vs 2B2P) 가스공급 분기</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>가스공급 준비 완료 후 상대측 공급 중일 때의 판정</t>
+        </is>
+      </c>
+      <c r="E16" s="18" t="inlineStr">
+        <is>
+          <t>GC Type: 2B1P(싱글포트) vs 2B2P(독립듀얼)</t>
+        </is>
+      </c>
+      <c r="F16" s="18" t="inlineStr">
+        <is>
+          <t>2B1P 시 반대편 가스공급 화면 자동 전환 / 2B2P 시 양측 동시 공급</t>
+        </is>
+      </c>
+      <c r="G16" s="18" t="inlineStr">
+        <is>
+          <t>하드웨어 타입 분기</t>
+        </is>
+      </c>
+      <c r="H16" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I16" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J16" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>[Step 01] IDLE 사전확인 7단계</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>실린더 잠금 Check 및 P&amp;ID 센서 정상 확인</t>
+        </is>
+      </c>
+      <c r="E17" s="18" t="inlineStr">
+        <is>
+          <t>Status: IDLE</t>
+        </is>
+      </c>
+      <c r="F17" s="18" t="inlineStr">
+        <is>
+          <t>사전확인 완료 ➔ Status 점멸 ➔ Puls 자동 인계</t>
+        </is>
+      </c>
+      <c r="G17" s="18" t="inlineStr">
+        <is>
+          <t>순차 파이프라인 1</t>
+        </is>
+      </c>
+      <c r="H17" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I17" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J17" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>[Step 02] Puls 잔류가스 제거</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>잔류가스 배기 및 Pulse Vent 시퀀스 진행</t>
+        </is>
+      </c>
+      <c r="E18" s="18" t="inlineStr">
+        <is>
+          <t>Status: Puls</t>
+        </is>
+      </c>
+      <c r="F18" s="18" t="inlineStr">
+        <is>
+          <t>Puls 완료 ➔ Status [1P]로 자동 인계</t>
+        </is>
+      </c>
+      <c r="G18" s="18" t="inlineStr">
+        <is>
+          <t>순차 파이프라인 2</t>
+        </is>
+      </c>
+      <c r="H18" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J18" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>[Step 03] 1P 1-2차측 Vent 및 퍼지</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>1P Vent ➔ 2차측 Purge ➔ Pumping ➔ 1차측 Purge</t>
+        </is>
+      </c>
+      <c r="E19" s="18" t="inlineStr">
+        <is>
+          <t>Status: 1P (4개 서브시퀀스 연속 체인)</t>
+        </is>
+      </c>
+      <c r="F19" s="18" t="inlineStr">
+        <is>
+          <t>1P 전 공정 완료 ➔ Status [-L]로 자동 인계</t>
+        </is>
+      </c>
+      <c r="G19" s="18" t="inlineStr">
+        <is>
+          <t>순차 파이프라인 3</t>
+        </is>
+      </c>
+      <c r="H19" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J19" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>[Step 04] -L 감압 및 누출 시험</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>진공 배기 후 감압 누출 압력 상승 감시</t>
+        </is>
+      </c>
+      <c r="E20" s="18" t="inlineStr">
+        <is>
+          <t>Status: -L</t>
+        </is>
+      </c>
+      <c r="F20" s="18" t="inlineStr">
+        <is>
+          <t>감압 합격 ➔ 옵션에 따라 (-VT 또는 2P)로 자동 인계</t>
+        </is>
+      </c>
+      <c r="G20" s="18" t="inlineStr">
+        <is>
+          <t>순차 파이프라인 4</t>
+        </is>
+      </c>
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J20" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>[Step 05] 2P 2차 배관청소</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>N2 퍼지 및 배관 진공 반복 청소</t>
+        </is>
+      </c>
+      <c r="E21" s="18" t="inlineStr">
+        <is>
+          <t>Status: 2P</t>
+        </is>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>2P 완료 ➔ 비밀번호 확인 ➔ [CC] 용기교체로 인계</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr">
+        <is>
+          <t>순차 파이프라인 5</t>
+        </is>
+      </c>
+      <c r="H21" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I21" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J21" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>[Step 06] CC 용기교체 6단계</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>용기 분리 ➔ 신규 용기 체결 ➔ 가스명/바코드 확인 ➔ 가드 닫힘</t>
+        </is>
+      </c>
+      <c r="E22" s="18" t="inlineStr">
+        <is>
+          <t>Status: CC</t>
+        </is>
+      </c>
+      <c r="F22" s="18" t="inlineStr">
+        <is>
+          <t>용기교체 확인 ➔ [3P] 3차 배관청소로 자동 인계</t>
+        </is>
+      </c>
+      <c r="G22" s="18" t="inlineStr">
+        <is>
+          <t>순차 파이프라인 6</t>
+        </is>
+      </c>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I22" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J22" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>[Step 07] 3P 3차 배관청소</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>신규 체결 배관 N2 퍼지 및 진공 청소</t>
+        </is>
+      </c>
+      <c r="E23" s="18" t="inlineStr">
+        <is>
+          <t>Status: 3P</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>3P 완료 ➔ [+L] 가압시험으로 자동 인계</t>
+        </is>
+      </c>
+      <c r="G23" s="18" t="inlineStr">
+        <is>
+          <t>순차 파이프라인 7</t>
+        </is>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I23" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J23" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>[Step 08] +L 가압시험 및 Puls 2</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>N2 고압 가압 누출 시험 ➔ Puls 2 잔류 배기</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Status: +L / Puls 2</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>+L 가압 합격 ➔ [4P] 4차 배관청소로 자동 인계</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>순차 파이프라인 8</t>
+        </is>
+      </c>
+      <c r="H24" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I24" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J24" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>[Step 09] 4P 4차 배관청소 및 PC 완료</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>최종 고순도 퍼지 ➔ 퍼지완료(PC) 전환</t>
+        </is>
+      </c>
+      <c r="E25" s="18" t="inlineStr">
+        <is>
+          <t>Status: 4P ➔ PC</t>
+        </is>
+      </c>
+      <c r="F25" s="18" t="inlineStr">
+        <is>
+          <t>PC 진입 ➔ 가스공급 메뉴 활성화 ➔ GSP 가스공급준비 인계</t>
+        </is>
+      </c>
+      <c r="G25" s="18" t="inlineStr">
+        <is>
+          <t>순차 파이프라인 9</t>
+        </is>
+      </c>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J25" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="17" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>[Step 10] GSP 가스공급준비 7단계</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>공급압력확인 ➔ 밸브셔터 ➔ 레귤레이터 ➔ 실린더Open ➔ FPV Open</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>가스공급 7단계 절차</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>가스공급준비 완료 ➔ Status [READY] 전환</t>
+        </is>
+      </c>
+      <c r="G26" s="18" t="inlineStr">
+        <is>
+          <t>순차 파이프라인 10</t>
+        </is>
+      </c>
+      <c r="H26" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I26" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J26" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>전구간체인</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>[Step 11] Service (가스공급 중) 최종 완주</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>최종 FPV 밸브 Open ➔ 정상 가스 공급 상태 도달</t>
+        </is>
+      </c>
+      <c r="E27" s="18" t="inlineStr">
+        <is>
+          <t>Status: Service (가스공급)</t>
+        </is>
+      </c>
+      <c r="F27" s="18" t="inlineStr">
+        <is>
+          <t>초기 IDLE부터 최종 Service까지 전 파이프라인 무중단 완주</t>
+        </is>
+      </c>
+      <c r="G27" s="18" t="inlineStr">
+        <is>
+          <t>최종 완료 안전 검증</t>
+        </is>
+      </c>
+      <c r="H27" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I27" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J27" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>녹화및산출물</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="inlineStr">
+        <is>
+          <t>실시간 화면 녹화 (Screen Record)</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>상단 [🎥 화면 녹화] 터치 ➔ 시뮬레이션 전과정 녹화 ➔ 저장</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>단말기 MP4 녹화</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>시뮬레이션 전과정 무손실 녹화 완료 및 파일 저장</t>
+        </is>
+      </c>
+      <c r="G28" s="18" t="inlineStr">
+        <is>
+          <t>운전자 검증 증적 확보</t>
+        </is>
+      </c>
+      <c r="H28" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I28" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J28" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>녹화및산출물</t>
+        </is>
+      </c>
+      <c r="C29" s="18" t="inlineStr">
+        <is>
+          <t>검증 체크시트 엑셀 자동 발행</t>
+        </is>
+      </c>
+      <c r="D29" s="18" t="inlineStr">
+        <is>
+          <t>시뮬레이션 완주 후 단말기 다운로드 폴더 자동 저장</t>
+        </is>
+      </c>
+      <c r="E29" s="18" t="inlineStr">
+        <is>
+          <t>엑셀 리포트 포맷</t>
+        </is>
+      </c>
+      <c r="F29" s="18" t="inlineStr">
+        <is>
+          <t>/storage/emulated/0/Download/GMS_...xlsx 자동 저장</t>
+        </is>
+      </c>
+      <c r="G29" s="18" t="inlineStr">
+        <is>
+          <t>품질 검증 보고서 발행</t>
+        </is>
+      </c>
+      <c r="H29" s="17" t="inlineStr">
+        <is>
+          <t>1x / 2x / 5x</t>
+        </is>
+      </c>
+      <c r="I29" s="17" t="inlineStr">
+        <is>
+          <t>자동 시뮬레이션 PASS</t>
+        </is>
+      </c>
+      <c r="J29" s="19" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:J29"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>